<commit_message>
Add IFRS-compliant Financial Notes with opening balances
- Add Opening Balance column to chart_of_accounts.xlsx
- Update coa_mapper.py to load opening balances from COA
- Add add_financial_notes_v3.py for IFRS-compliant Financial Notes
  - Shows Opening/Movement/Closing columns from Trial Balance
  - Removes accumulated depreciation from Balance Sheet face
  - Assets shown at Net Book Value (IFRS compliant)
- Update batch_process_all_months.py for correct opening balance handling
- Regenerate all output files for Feb-Oct 2025
- All 9 months pass Module 7 validation (Assets = Equity + Liabilities)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/accountant-skill/data/input/master/chart_of_accounts.xlsx
+++ b/accountant-skill/data/input/master/chart_of_accounts.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Opening Balance</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -567,6 +572,9 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="G5" t="n">
+        <v>5605177</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -597,6 +605,9 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="G6" t="n">
+        <v>7899300</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -627,6 +638,9 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="G7" t="n">
+        <v>34461646</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -777,6 +791,9 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="G12" t="n">
+        <v>219000000</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -807,6 +824,9 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="G13" t="n">
+        <v>133000000</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -837,6 +857,9 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="G14" t="n">
+        <v>19950000</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -867,6 +890,9 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="G15" t="n">
+        <v>66400000</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -897,6 +923,9 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="G16" t="n">
+        <v>12375300</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -987,6 +1016,9 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="G19" t="n">
+        <v>7200000</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1017,6 +1049,9 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="G20" t="n">
+        <v>1710000</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1316,6 +1351,9 @@
         <is>
           <t>Active</t>
         </is>
+      </c>
+      <c r="G30" t="n">
+        <v>439530823</v>
       </c>
     </row>
     <row r="31">

</xml_diff>